<commit_message>
feat: risk tablosunun altina Diger (35. faktor) aciklama dipnotu eklendi (UI, Excel, Word, HTML)
</commit_message>
<xml_diff>
--- a/exports/Guncel_8B_Sinif_Risk_Haritasi.xlsx
+++ b/exports/Guncel_8B_Sinif_Risk_Haritasi.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,6 +58,19 @@
       <b val="1"/>
       <color rgb="00C00000"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="001F497D"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00404040"/>
+      <sz val="8.5"/>
     </font>
   </fonts>
   <fills count="7">
@@ -138,7 +151,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -183,6 +196,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -548,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM34"/>
+  <dimension ref="A1:AM37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.5" customWidth="1" min="1" max="1"/>
@@ -2744,11 +2763,27 @@
         <v>40</v>
       </c>
     </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t>📌 35. FAKTÖR ('DİĞER') AÇIKLAMASI: İlk 34 standart MEB risk kategorisinde yer almayan; ancak öğrencinin akademik ve psikososyal takibini gerektiren özel durumları ifade eder (Ağır sınav kaygısı, son 1-2 yılda yaşanan travmatik/önemli olaylar, duygusal tükenmişlik veya öğrencinin bildirdiği özel güçlükler).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="17" t="inlineStr">
+        <is>
+          <t>* 8/B Sınıfı 'Diğer' Kapsamındaki Durumlar: Melek Rana Kesici ('yaşamak' - psikososyal takip), Halit Eren Hatunoğlu ('kaygı'), Derin Yılmaz (önemli ailevi olay), Meryem Bozdemir (önemli ailevi olay), Tuna Koç (akran uyumu), Sümeyye Taşkın &amp; Beren Koç (ulaşım problemi).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
+    <mergeCell ref="A37:AM37"/>
+    <mergeCell ref="A2:AL2"/>
     <mergeCell ref="A1:AL1"/>
     <mergeCell ref="A34:C34"/>
-    <mergeCell ref="A2:AL2"/>
+    <mergeCell ref="A36:AM36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>